<commit_message>
Geração e Envio de QrCodes Revisados, Nova Branch Criada
</commit_message>
<xml_diff>
--- a/QRsend1366/src/dados.xlsx
+++ b/QRsend1366/src/dados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,18 +431,10 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11 964440570</t>
+          <t>11 983787869</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>11 983787869</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Criação de Metodo de Envio de Parceeiro (QrList)
</commit_message>
<xml_diff>
--- a/QRsend1366/src/dados.xlsx
+++ b/QRsend1366/src/dados.xlsx
@@ -429,10 +429,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>11 983787869</t>
-        </is>
+      <c r="A2" t="n">
+        <v>11983787869</v>
       </c>
       <c r="B2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Script de Envio /  Imagens da WEB
</commit_message>
<xml_diff>
--- a/QRsend1366/src/dados.xlsx
+++ b/QRsend1366/src/dados.xlsx
@@ -429,8 +429,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>11983787869</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>11 983787869</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr"/>
     </row>

</xml_diff>